<commit_message>
Mode prospectif équilibré ! Reste à se pencher sur les problèmes d'allocation de la fertilisation synthétique
</commit_message>
<xml_diff>
--- a/example/GRAFS_data_example_C_prospect.xlsx
+++ b/example/GRAFS_data_example_C_prospect.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3DE6695-457C-4943-B968-640287EF76B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A475F1-12D7-4924-BC7F-8E74CEE21757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16530" yWindow="-15870" windowWidth="25440" windowHeight="15270" xr2:uid="{F475FEA0-B9E5-4A03-9EDE-4A3E6C5C262C}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="89">
   <si>
     <t>Area</t>
   </si>
@@ -854,7 +854,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5D825A9-0C1C-44E4-98B7-F194F26ABDB6}">
-  <dimension ref="A1:E176"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.36328125" customWidth="1"/>
@@ -2994,7 +2994,7 @@
         <v>5</v>
       </c>
       <c r="B126">
-        <v>1961</v>
+        <v>2023</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>35</v>
@@ -3003,7 +3003,7 @@
         <v>41</v>
       </c>
       <c r="E126">
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.35">
@@ -3011,16 +3011,16 @@
         <v>5</v>
       </c>
       <c r="B127">
-        <v>2023</v>
+        <v>1961</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E127">
-        <v>300</v>
+        <v>50</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.35">
@@ -3028,7 +3028,7 @@
         <v>5</v>
       </c>
       <c r="B128">
-        <v>1961</v>
+        <v>2023</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>35</v>
@@ -3037,7 +3037,7 @@
         <v>42</v>
       </c>
       <c r="E128">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.35">
@@ -3045,16 +3045,16 @@
         <v>5</v>
       </c>
       <c r="B129">
-        <v>2023</v>
+        <v>1961</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E129">
-        <v>70</v>
+        <v>8</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.35">
@@ -3062,7 +3062,7 @@
         <v>5</v>
       </c>
       <c r="B130">
-        <v>1961</v>
+        <v>2023</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>35</v>
@@ -3085,10 +3085,10 @@
         <v>35</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E131">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.35">
@@ -3102,10 +3102,10 @@
         <v>35</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E132">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.35">
@@ -3119,10 +3119,10 @@
         <v>35</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E133">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.35">
@@ -3130,16 +3130,16 @@
         <v>5</v>
       </c>
       <c r="B134">
-        <v>2023</v>
+        <v>1961</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E134">
-        <v>0.05</v>
+        <v>61</v>
+      </c>
+      <c r="E134" s="1" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.35">
@@ -3147,7 +3147,7 @@
         <v>5</v>
       </c>
       <c r="B135">
-        <v>1961</v>
+        <v>2023</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>35</v>
@@ -3156,7 +3156,7 @@
         <v>61</v>
       </c>
       <c r="E135" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.35">
@@ -3167,13 +3167,13 @@
         <v>2023</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D136" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E136" s="1" t="s">
-        <v>63</v>
+        <v>25</v>
+      </c>
+      <c r="D136" t="s">
+        <v>14</v>
+      </c>
+      <c r="E136" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.35">
@@ -3187,10 +3187,10 @@
         <v>25</v>
       </c>
       <c r="D137" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E137" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.35">
@@ -3204,10 +3204,10 @@
         <v>25</v>
       </c>
       <c r="D138" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E138" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.35">
@@ -3215,16 +3215,16 @@
         <v>5</v>
       </c>
       <c r="B139">
-        <v>2023</v>
+        <v>1961</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>25</v>
       </c>
       <c r="D139" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E139" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.35">
@@ -3238,10 +3238,10 @@
         <v>25</v>
       </c>
       <c r="D140" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E140" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.35">
@@ -3255,27 +3255,27 @@
         <v>25</v>
       </c>
       <c r="D141" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E141" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A142" s="1" t="s">
+      <c r="A142" t="s">
         <v>5</v>
       </c>
       <c r="B142">
         <v>1961</v>
       </c>
-      <c r="C142" s="1" t="s">
+      <c r="C142" t="s">
         <v>25</v>
       </c>
       <c r="D142" t="s">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="E142" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.35">
@@ -3283,7 +3283,7 @@
         <v>5</v>
       </c>
       <c r="B143">
-        <v>1961</v>
+        <v>2023</v>
       </c>
       <c r="C143" t="s">
         <v>25</v>
@@ -3296,155 +3296,155 @@
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A144" t="s">
-        <v>5</v>
-      </c>
-      <c r="B144">
-        <v>2023</v>
-      </c>
-      <c r="C144" t="s">
-        <v>25</v>
-      </c>
-      <c r="D144" t="s">
-        <v>80</v>
-      </c>
-      <c r="E144" t="s">
-        <v>76</v>
+      <c r="A144" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B144" s="2">
+        <v>1961</v>
+      </c>
+      <c r="C144" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D144" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E144" s="8">
+        <v>2.76</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A145" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B145" s="2">
-        <v>1961</v>
-      </c>
-      <c r="C145" s="5" t="s">
+      <c r="A145" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B145" s="3">
+        <v>1961</v>
+      </c>
+      <c r="C145" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D145" s="5" t="s">
-        <v>59</v>
+      <c r="D145" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="E145" s="8">
-        <v>2.76</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A146" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B146" s="3">
-        <v>1961</v>
-      </c>
-      <c r="C146" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D146" s="6" t="s">
-        <v>52</v>
+      <c r="A146" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B146" s="2">
+        <v>1961</v>
+      </c>
+      <c r="C146" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D146" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="E146" s="8">
-        <v>1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A147" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B147" s="2">
+      <c r="A147" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B147" s="3">
         <v>1961</v>
       </c>
       <c r="C147" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D147" s="5" t="s">
-        <v>6</v>
+      <c r="D147" s="6" t="s">
+        <v>58</v>
       </c>
       <c r="E147" s="8">
-        <v>2.5</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A148" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B148" s="3">
+      <c r="A148" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B148" s="2">
         <v>1961</v>
       </c>
       <c r="C148" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D148" s="6" t="s">
-        <v>58</v>
+      <c r="D148" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="E148" s="8">
         <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A149" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B149" s="2">
+      <c r="A149" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B149" s="3">
         <v>1961</v>
       </c>
       <c r="C149" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D149" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E149" s="8">
-        <v>2.2000000000000002</v>
+      <c r="D149" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E149" s="4">
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A150" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B150" s="3">
+      <c r="A150" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B150" s="2">
         <v>1961</v>
       </c>
       <c r="C150" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D150" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E150" s="4">
-        <v>0</v>
+      <c r="D150" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E150" s="8">
+        <v>3.5</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A151" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B151" s="2">
+      <c r="A151" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B151" s="3">
         <v>1961</v>
       </c>
       <c r="C151" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D151" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E151" s="8">
-        <v>3.5</v>
+      <c r="D151" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E151" s="11">
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A152" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B152" s="3">
+      <c r="A152" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B152" s="2">
         <v>1961</v>
       </c>
       <c r="C152" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D152" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E152" s="11">
+      <c r="D152" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E152" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3453,117 +3453,117 @@
         <v>5</v>
       </c>
       <c r="B153" s="2">
-        <v>1961</v>
+        <v>2023</v>
       </c>
       <c r="C153" s="5" t="s">
         <v>33</v>
       </c>
       <c r="D153" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E153" s="12">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="E153" s="8">
+        <v>2.5</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A154" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B154" s="2">
+      <c r="A154" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B154" s="3">
         <v>2023</v>
       </c>
       <c r="C154" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D154" s="5" t="s">
-        <v>6</v>
+      <c r="D154" s="6" t="s">
+        <v>58</v>
       </c>
       <c r="E154" s="8">
-        <v>2.5</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A155" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B155" s="3">
+      <c r="A155" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B155" s="2">
         <v>2023</v>
       </c>
       <c r="C155" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D155" s="6" t="s">
-        <v>58</v>
+      <c r="D155" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="E155" s="8">
         <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A156" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B156" s="2">
+      <c r="A156" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B156" s="3">
         <v>2023</v>
       </c>
       <c r="C156" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D156" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E156" s="8">
-        <v>2.2000000000000002</v>
+      <c r="D156" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E156" s="4">
+        <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A157" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B157" s="3">
+      <c r="A157" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B157" s="2">
         <v>2023</v>
       </c>
       <c r="C157" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D157" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E157" s="4">
-        <v>0</v>
+      <c r="D157" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E157" s="8">
+        <v>3.5</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A158" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B158" s="2">
+      <c r="A158" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B158" s="3">
         <v>2023</v>
       </c>
       <c r="C158" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D158" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E158" s="8">
-        <v>3.5</v>
+      <c r="D158" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E158" s="11">
+        <v>0</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A159" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B159" s="3">
+      <c r="A159" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B159" s="2">
         <v>2023</v>
       </c>
       <c r="C159" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D159" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E159" s="11">
+      <c r="D159" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E159" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3572,118 +3572,118 @@
         <v>5</v>
       </c>
       <c r="B160" s="2">
-        <v>2023</v>
+        <v>1961</v>
       </c>
       <c r="C160" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D160" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E160" s="12">
+        <v>6</v>
+      </c>
+      <c r="E160">
         <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A161" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B161" s="2">
+      <c r="A161" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B161" s="3">
         <v>1961</v>
       </c>
       <c r="C161" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D161" s="5" t="s">
-        <v>6</v>
+      <c r="D161" s="6" t="s">
+        <v>58</v>
       </c>
       <c r="E161">
         <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A162" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B162" s="3">
+      <c r="A162" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B162" s="2">
         <v>1961</v>
       </c>
       <c r="C162" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D162" s="6" t="s">
-        <v>58</v>
+      <c r="D162" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="E162">
         <v>0</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A163" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B163" s="2">
+      <c r="A163" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B163" s="3">
         <v>1961</v>
       </c>
       <c r="C163" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D163" s="5" t="s">
-        <v>7</v>
+      <c r="D163" s="6" t="s">
+        <v>8</v>
       </c>
       <c r="E163">
-        <v>0</v>
+        <v>125</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A164" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B164" s="3">
+      <c r="A164" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B164" s="2">
         <v>1961</v>
       </c>
       <c r="C164" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D164" s="6" t="s">
-        <v>8</v>
+      <c r="D164" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="E164">
-        <v>125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A165" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B165" s="2">
+      <c r="A165" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B165" s="3">
         <v>1961</v>
       </c>
       <c r="C165" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D165" s="5" t="s">
-        <v>9</v>
+      <c r="D165" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="E165">
         <v>0</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A166" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B166" s="3">
+      <c r="A166" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B166" s="2">
         <v>1961</v>
       </c>
       <c r="C166" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D166" s="6" t="s">
-        <v>11</v>
+      <c r="D166" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="E166">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.35">
@@ -3691,135 +3691,135 @@
         <v>5</v>
       </c>
       <c r="B167" s="2">
-        <v>1961</v>
+        <v>2023</v>
       </c>
       <c r="C167" s="5" t="s">
         <v>34</v>
       </c>
       <c r="D167" s="5" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E167">
-        <v>150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A168" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B168" s="2">
+      <c r="A168" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B168" s="3">
         <v>2023</v>
       </c>
       <c r="C168" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D168" s="5" t="s">
-        <v>6</v>
+      <c r="D168" s="6" t="s">
+        <v>58</v>
       </c>
       <c r="E168">
         <v>0</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A169" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B169" s="3">
+      <c r="A169" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B169" s="2">
         <v>2023</v>
       </c>
       <c r="C169" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D169" s="6" t="s">
-        <v>58</v>
+      <c r="D169" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="E169">
         <v>0</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A170" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B170" s="2">
+      <c r="A170" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B170" s="3">
         <v>2023</v>
       </c>
       <c r="C170" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D170" s="5" t="s">
-        <v>7</v>
+      <c r="D170" s="6" t="s">
+        <v>8</v>
       </c>
       <c r="E170">
-        <v>0</v>
+        <v>125</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A171" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B171" s="3">
+      <c r="A171" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B171" s="2">
         <v>2023</v>
       </c>
       <c r="C171" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D171" s="6" t="s">
-        <v>8</v>
+      <c r="D171" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="E171">
-        <v>125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A172" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B172" s="2">
+      <c r="A172" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B172" s="3">
         <v>2023</v>
       </c>
       <c r="C172" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D172" s="5" t="s">
-        <v>9</v>
+      <c r="D172" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="E172">
         <v>0</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A173" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B173" s="3">
+      <c r="A173" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B173" s="2">
         <v>2023</v>
       </c>
       <c r="C173" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D173" s="6" t="s">
-        <v>11</v>
+      <c r="D173" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="E173">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A174" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B174" s="2">
-        <v>2023</v>
-      </c>
-      <c r="C174" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D174" s="5" t="s">
-        <v>22</v>
+      <c r="A174" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B174" s="14">
+        <v>1961</v>
+      </c>
+      <c r="C174" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D174" t="s">
+        <v>39</v>
       </c>
       <c r="E174">
-        <v>150</v>
+        <v>20</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.35">
@@ -3827,7 +3827,7 @@
         <v>5</v>
       </c>
       <c r="B175" s="14">
-        <v>1961</v>
+        <v>2023</v>
       </c>
       <c r="C175" s="15" t="s">
         <v>12</v>
@@ -3836,23 +3836,6 @@
         <v>39</v>
       </c>
       <c r="E175">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A176" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="B176" s="14">
-        <v>2023</v>
-      </c>
-      <c r="C176" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D176" t="s">
-        <v>39</v>
-      </c>
-      <c r="E176">
         <v>25</v>
       </c>
     </row>

</xml_diff>